<commit_message>
feat: redesign KPI cards — full-width premium layout with gradient accents, icons, and delete action
</commit_message>
<xml_diff>
--- a/test_data.xlsx
+++ b/test_data.xlsx
@@ -418,10 +418,10 @@
         <v>A</v>
       </c>
       <c r="B2">
-        <v>630</v>
+        <v>322</v>
       </c>
       <c r="C2">
-        <v>-4</v>
+        <v>-48</v>
       </c>
       <c r="D2" t="str">
         <v>2022-12-31</v>
@@ -432,10 +432,10 @@
         <v>B</v>
       </c>
       <c r="B3">
-        <v>218</v>
+        <v>612</v>
       </c>
       <c r="C3">
-        <v>177</v>
+        <v>138</v>
       </c>
       <c r="D3" t="str">
         <v>2023-01-01</v>
@@ -446,10 +446,10 @@
         <v>C</v>
       </c>
       <c r="B4">
-        <v>622</v>
+        <v>301</v>
       </c>
       <c r="C4">
-        <v>52</v>
+        <v>193</v>
       </c>
       <c r="D4" t="str">
         <v>2023-01-02</v>
@@ -460,10 +460,10 @@
         <v>D</v>
       </c>
       <c r="B5">
-        <v>588</v>
+        <v>558</v>
       </c>
       <c r="C5">
-        <v>180</v>
+        <v>120</v>
       </c>
       <c r="D5" t="str">
         <v>2023-01-03</v>
@@ -474,10 +474,10 @@
         <v>A</v>
       </c>
       <c r="B6">
-        <v>440</v>
+        <v>401</v>
       </c>
       <c r="C6">
-        <v>-23</v>
+        <v>129</v>
       </c>
       <c r="D6" t="str">
         <v>2023-01-04</v>
@@ -488,10 +488,10 @@
         <v>B</v>
       </c>
       <c r="B7">
-        <v>269</v>
+        <v>595</v>
       </c>
       <c r="C7">
-        <v>7</v>
+        <v>134</v>
       </c>
       <c r="D7" t="str">
         <v>2023-01-05</v>
@@ -502,10 +502,10 @@
         <v>C</v>
       </c>
       <c r="B8">
-        <v>954</v>
+        <v>809</v>
       </c>
       <c r="C8">
-        <v>71</v>
+        <v>142</v>
       </c>
       <c r="D8" t="str">
         <v>2023-01-06</v>
@@ -516,10 +516,10 @@
         <v>D</v>
       </c>
       <c r="B9">
-        <v>306</v>
+        <v>249</v>
       </c>
       <c r="C9">
-        <v>68</v>
+        <v>-11</v>
       </c>
       <c r="D9" t="str">
         <v>2023-01-07</v>
@@ -530,10 +530,10 @@
         <v>A</v>
       </c>
       <c r="B10">
-        <v>403</v>
+        <v>584</v>
       </c>
       <c r="C10">
-        <v>33</v>
+        <v>74</v>
       </c>
       <c r="D10" t="str">
         <v>2023-01-08</v>
@@ -544,10 +544,10 @@
         <v>B</v>
       </c>
       <c r="B11">
-        <v>247</v>
+        <v>749</v>
       </c>
       <c r="C11">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="D11" t="str">
         <v>2023-01-09</v>
@@ -558,10 +558,10 @@
         <v>C</v>
       </c>
       <c r="B12">
-        <v>705</v>
+        <v>814</v>
       </c>
       <c r="C12">
-        <v>46</v>
+        <v>119</v>
       </c>
       <c r="D12" t="str">
         <v>2023-01-10</v>
@@ -572,10 +572,10 @@
         <v>D</v>
       </c>
       <c r="B13">
-        <v>852</v>
+        <v>123</v>
       </c>
       <c r="C13">
-        <v>99</v>
+        <v>64</v>
       </c>
       <c r="D13" t="str">
         <v>2023-01-11</v>
@@ -586,10 +586,10 @@
         <v>A</v>
       </c>
       <c r="B14">
-        <v>342</v>
+        <v>404</v>
       </c>
       <c r="C14">
-        <v>134</v>
+        <v>-47</v>
       </c>
       <c r="D14" t="str">
         <v>2023-01-12</v>
@@ -600,10 +600,10 @@
         <v>B</v>
       </c>
       <c r="B15">
-        <v>680</v>
+        <v>900</v>
       </c>
       <c r="C15">
-        <v>32</v>
+        <v>-47</v>
       </c>
       <c r="D15" t="str">
         <v>2023-01-13</v>
@@ -614,10 +614,10 @@
         <v>C</v>
       </c>
       <c r="B16">
-        <v>256</v>
+        <v>446</v>
       </c>
       <c r="C16">
-        <v>110</v>
+        <v>22</v>
       </c>
       <c r="D16" t="str">
         <v>2023-01-14</v>
@@ -628,10 +628,10 @@
         <v>D</v>
       </c>
       <c r="B17">
-        <v>741</v>
+        <v>590</v>
       </c>
       <c r="C17">
-        <v>73</v>
+        <v>-31</v>
       </c>
       <c r="D17" t="str">
         <v>2023-01-15</v>
@@ -642,10 +642,10 @@
         <v>A</v>
       </c>
       <c r="B18">
-        <v>875</v>
+        <v>578</v>
       </c>
       <c r="C18">
-        <v>17</v>
+        <v>-16</v>
       </c>
       <c r="D18" t="str">
         <v>2023-01-16</v>
@@ -656,10 +656,10 @@
         <v>B</v>
       </c>
       <c r="B19">
-        <v>159</v>
+        <v>630</v>
       </c>
       <c r="C19">
-        <v>62</v>
+        <v>111</v>
       </c>
       <c r="D19" t="str">
         <v>2023-01-17</v>
@@ -670,10 +670,10 @@
         <v>C</v>
       </c>
       <c r="B20">
-        <v>760</v>
+        <v>504</v>
       </c>
       <c r="C20">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="D20" t="str">
         <v>2023-01-18</v>
@@ -684,10 +684,10 @@
         <v>D</v>
       </c>
       <c r="B21">
-        <v>215</v>
+        <v>411</v>
       </c>
       <c r="C21">
-        <v>13</v>
+        <v>196</v>
       </c>
       <c r="D21" t="str">
         <v>2023-01-19</v>
@@ -698,10 +698,10 @@
         <v>A</v>
       </c>
       <c r="B22">
-        <v>575</v>
+        <v>324</v>
       </c>
       <c r="C22">
-        <v>85</v>
+        <v>178</v>
       </c>
       <c r="D22" t="str">
         <v>2023-01-20</v>
@@ -712,10 +712,10 @@
         <v>B</v>
       </c>
       <c r="B23">
-        <v>341</v>
+        <v>729</v>
       </c>
       <c r="C23">
-        <v>54</v>
+        <v>-28</v>
       </c>
       <c r="D23" t="str">
         <v>2023-01-21</v>
@@ -726,10 +726,10 @@
         <v>C</v>
       </c>
       <c r="B24">
-        <v>790</v>
+        <v>952</v>
       </c>
       <c r="C24">
-        <v>69</v>
+        <v>-1</v>
       </c>
       <c r="D24" t="str">
         <v>2023-01-22</v>
@@ -740,10 +740,10 @@
         <v>D</v>
       </c>
       <c r="B25">
-        <v>705</v>
+        <v>643</v>
       </c>
       <c r="C25">
-        <v>103</v>
+        <v>10</v>
       </c>
       <c r="D25" t="str">
         <v>2023-01-23</v>
@@ -754,10 +754,10 @@
         <v>A</v>
       </c>
       <c r="B26">
-        <v>648</v>
+        <v>129</v>
       </c>
       <c r="C26">
-        <v>-46</v>
+        <v>194</v>
       </c>
       <c r="D26" t="str">
         <v>2023-01-24</v>
@@ -768,10 +768,10 @@
         <v>B</v>
       </c>
       <c r="B27">
-        <v>426</v>
+        <v>468</v>
       </c>
       <c r="C27">
-        <v>177</v>
+        <v>84</v>
       </c>
       <c r="D27" t="str">
         <v>2023-01-25</v>
@@ -782,10 +782,10 @@
         <v>C</v>
       </c>
       <c r="B28">
-        <v>301</v>
+        <v>842</v>
       </c>
       <c r="C28">
-        <v>159</v>
+        <v>31</v>
       </c>
       <c r="D28" t="str">
         <v>2023-01-26</v>
@@ -796,10 +796,10 @@
         <v>D</v>
       </c>
       <c r="B29">
-        <v>282</v>
+        <v>167</v>
       </c>
       <c r="C29">
-        <v>119</v>
+        <v>80</v>
       </c>
       <c r="D29" t="str">
         <v>2023-01-27</v>
@@ -810,10 +810,10 @@
         <v>A</v>
       </c>
       <c r="B30">
-        <v>560</v>
+        <v>636</v>
       </c>
       <c r="C30">
-        <v>-36</v>
+        <v>78</v>
       </c>
       <c r="D30" t="str">
         <v>2023-01-28</v>
@@ -824,10 +824,10 @@
         <v>B</v>
       </c>
       <c r="B31">
-        <v>766</v>
+        <v>216</v>
       </c>
       <c r="C31">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="D31" t="str">
         <v>2023-01-29</v>
@@ -838,10 +838,10 @@
         <v>C</v>
       </c>
       <c r="B32">
-        <v>354</v>
+        <v>281</v>
       </c>
       <c r="C32">
-        <v>-28</v>
+        <v>39</v>
       </c>
       <c r="D32" t="str">
         <v>2022-12-31</v>
@@ -852,10 +852,10 @@
         <v>D</v>
       </c>
       <c r="B33">
-        <v>932</v>
+        <v>462</v>
       </c>
       <c r="C33">
-        <v>-40</v>
+        <v>73</v>
       </c>
       <c r="D33" t="str">
         <v>2023-01-01</v>
@@ -866,10 +866,10 @@
         <v>A</v>
       </c>
       <c r="B34">
-        <v>241</v>
+        <v>169</v>
       </c>
       <c r="C34">
-        <v>185</v>
+        <v>-11</v>
       </c>
       <c r="D34" t="str">
         <v>2023-01-02</v>
@@ -880,10 +880,10 @@
         <v>B</v>
       </c>
       <c r="B35">
-        <v>223</v>
+        <v>144</v>
       </c>
       <c r="C35">
-        <v>65</v>
+        <v>132</v>
       </c>
       <c r="D35" t="str">
         <v>2023-01-03</v>
@@ -894,10 +894,10 @@
         <v>C</v>
       </c>
       <c r="B36">
-        <v>727</v>
+        <v>260</v>
       </c>
       <c r="C36">
-        <v>-5</v>
+        <v>65</v>
       </c>
       <c r="D36" t="str">
         <v>2023-01-04</v>
@@ -908,10 +908,10 @@
         <v>D</v>
       </c>
       <c r="B37">
-        <v>984</v>
+        <v>406</v>
       </c>
       <c r="C37">
-        <v>-30</v>
+        <v>32</v>
       </c>
       <c r="D37" t="str">
         <v>2023-01-05</v>
@@ -922,10 +922,10 @@
         <v>A</v>
       </c>
       <c r="B38">
-        <v>955</v>
+        <v>536</v>
       </c>
       <c r="C38">
-        <v>67</v>
+        <v>195</v>
       </c>
       <c r="D38" t="str">
         <v>2023-01-06</v>
@@ -936,10 +936,10 @@
         <v>B</v>
       </c>
       <c r="B39">
-        <v>117</v>
+        <v>872</v>
       </c>
       <c r="C39">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="D39" t="str">
         <v>2023-01-07</v>
@@ -950,10 +950,10 @@
         <v>C</v>
       </c>
       <c r="B40">
-        <v>860</v>
+        <v>438</v>
       </c>
       <c r="C40">
-        <v>15</v>
+        <v>45</v>
       </c>
       <c r="D40" t="str">
         <v>2023-01-08</v>
@@ -964,10 +964,10 @@
         <v>D</v>
       </c>
       <c r="B41">
-        <v>879</v>
+        <v>189</v>
       </c>
       <c r="C41">
-        <v>-12</v>
+        <v>110</v>
       </c>
       <c r="D41" t="str">
         <v>2023-01-09</v>
@@ -978,10 +978,10 @@
         <v>A</v>
       </c>
       <c r="B42">
-        <v>548</v>
+        <v>228</v>
       </c>
       <c r="C42">
-        <v>72</v>
+        <v>4</v>
       </c>
       <c r="D42" t="str">
         <v>2023-01-10</v>
@@ -992,10 +992,10 @@
         <v>B</v>
       </c>
       <c r="B43">
-        <v>297</v>
+        <v>616</v>
       </c>
       <c r="C43">
-        <v>154</v>
+        <v>33</v>
       </c>
       <c r="D43" t="str">
         <v>2023-01-11</v>
@@ -1006,10 +1006,10 @@
         <v>C</v>
       </c>
       <c r="B44">
-        <v>948</v>
+        <v>580</v>
       </c>
       <c r="C44">
-        <v>22</v>
+        <v>107</v>
       </c>
       <c r="D44" t="str">
         <v>2023-01-12</v>
@@ -1020,10 +1020,10 @@
         <v>D</v>
       </c>
       <c r="B45">
-        <v>322</v>
+        <v>687</v>
       </c>
       <c r="C45">
-        <v>22</v>
+        <v>171</v>
       </c>
       <c r="D45" t="str">
         <v>2023-01-13</v>
@@ -1034,10 +1034,10 @@
         <v>A</v>
       </c>
       <c r="B46">
-        <v>224</v>
+        <v>751</v>
       </c>
       <c r="C46">
-        <v>171</v>
+        <v>112</v>
       </c>
       <c r="D46" t="str">
         <v>2023-01-14</v>
@@ -1048,10 +1048,10 @@
         <v>B</v>
       </c>
       <c r="B47">
-        <v>876</v>
+        <v>500</v>
       </c>
       <c r="C47">
-        <v>13</v>
+        <v>91</v>
       </c>
       <c r="D47" t="str">
         <v>2023-01-15</v>
@@ -1062,10 +1062,10 @@
         <v>C</v>
       </c>
       <c r="B48">
-        <v>141</v>
+        <v>685</v>
       </c>
       <c r="C48">
-        <v>51</v>
+        <v>143</v>
       </c>
       <c r="D48" t="str">
         <v>2023-01-16</v>
@@ -1076,10 +1076,10 @@
         <v>D</v>
       </c>
       <c r="B49">
-        <v>784</v>
+        <v>958</v>
       </c>
       <c r="C49">
-        <v>16</v>
+        <v>52</v>
       </c>
       <c r="D49" t="str">
         <v>2023-01-17</v>
@@ -1090,10 +1090,10 @@
         <v>A</v>
       </c>
       <c r="B50">
-        <v>358</v>
+        <v>913</v>
       </c>
       <c r="C50">
-        <v>128</v>
+        <v>85</v>
       </c>
       <c r="D50" t="str">
         <v>2023-01-18</v>
@@ -1104,10 +1104,10 @@
         <v>B</v>
       </c>
       <c r="B51">
-        <v>241</v>
+        <v>261</v>
       </c>
       <c r="C51">
-        <v>175</v>
+        <v>56</v>
       </c>
       <c r="D51" t="str">
         <v>2023-01-19</v>

</xml_diff>